<commit_message>
Refactor code structure and remove redundant sections for improved readability and maintainability
</commit_message>
<xml_diff>
--- a/output/admin-reporting/all-reports.xlsx
+++ b/output/admin-reporting/all-reports.xlsx
@@ -38,8 +38,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="true">Templates!$A$6:$L$8</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">Templates!$A$1:$L$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">Subscriptions!$A:$B,Subscriptions!$6:$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="true">Subscriptions!$A$6:$Q$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">Subscriptions!$A$1:$Q$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="true">Subscriptions!$A$6:$R$9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">Subscriptions!$A$1:$R$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">Engagement!$A:$B,Engagement!$6:$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="true">Engagement!$A$6:$S$9</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">Engagement!$A$1:$S$9</definedName>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="N7" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="N8" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="N9" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="N10" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
       </c>
       <c r="N11" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="N12" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="N13" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="N14" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1878,7 @@
       </c>
       <c r="N15" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="N16" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="N17" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="N18" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="N19" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="N20" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="N21" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2368,7 @@
       </c>
       <c r="N22" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="N23" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2508,7 @@
       </c>
       <c r="N24" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="N25" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2648,7 +2648,7 @@
       </c>
       <c r="N26" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="N27" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="N28" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="N29" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2928,7 @@
       </c>
       <c r="N30" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="N31" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -3068,7 +3068,7 @@
       </c>
       <c r="N32" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="N33" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="N34" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -3538,7 +3538,7 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C58" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -5177,7 +5177,7 @@
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -5819,7 +5819,7 @@
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -6140,7 +6140,7 @@
       </c>
       <c r="C172" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -6461,7 +6461,7 @@
       </c>
       <c r="C191" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15.1</t>
+          <t>2026-10-24.1</t>
         </is>
       </c>
     </row>
@@ -10293,7 +10293,7 @@
       </c>
       <c r="I7" s="1" t="inlineStr">
         <is>
-          <t>Unavailable / មិនមានទិន្នន័យ</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="J7" s="1" t="inlineStr">
@@ -10620,7 +10620,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="8.0" customWidth="true"/>
@@ -10638,8 +10638,9 @@
     <col min="13" max="13" width="17.0" customWidth="true"/>
     <col min="14" max="14" width="27.0" customWidth="true"/>
     <col min="15" max="15" width="27.0" customWidth="true"/>
-    <col min="16" max="16" width="23.0" customWidth="true"/>
+    <col min="16" max="16" width="27.0" customWidth="true"/>
     <col min="17" max="17" width="23.0" customWidth="true"/>
+    <col min="18" max="18" width="23.0" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" ht="38.0">
@@ -10762,11 +10763,17 @@
       </c>
       <c r="P6" s="7" t="inlineStr">
         <is>
+          <t>ប្រភពសិទ្ធិ
+Entitlement source</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="inlineStr">
+        <is>
           <t>ថ្ងៃទូទាត់
 Paid at</t>
         </is>
       </c>
-      <c r="Q6" s="7" t="inlineStr">
+      <c r="R6" s="7" t="inlineStr">
         <is>
           <t>ថ្ងៃបង្កើត
 Created at</t>
@@ -10844,7 +10851,12 @@
           <t>Unavailable / មិនមានទិន្នន័យ</t>
         </is>
       </c>
-      <c r="Q7" s="6" t="n">
+      <c r="Q7" s="1" t="inlineStr">
+        <is>
+          <t>Unavailable / មិនមានទិន្នន័យ</t>
+        </is>
+      </c>
+      <c r="R7" s="6" t="n">
         <v>46310.291666666664</v>
       </c>
     </row>
@@ -10910,10 +10922,15 @@
           <t>ABA</t>
         </is>
       </c>
-      <c r="P8" s="6" t="n">
+      <c r="P8" s="1" t="inlineStr">
+        <is>
+          <t>TELEGRAM_ADMIN_DETECT</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="n">
         <v>46310.333333333336</v>
       </c>
-      <c r="Q8" s="6" t="n">
+      <c r="R8" s="6" t="n">
         <v>46310.291666666664</v>
       </c>
     </row>
@@ -10977,20 +10994,25 @@
           <t>ABA</t>
         </is>
       </c>
-      <c r="P9" s="6" t="n">
+      <c r="P9" s="1" t="inlineStr">
+        <is>
+          <t>MANUAL_ADMIN</t>
+        </is>
+      </c>
+      <c r="Q9" s="6" t="n">
         <v>46310.333333333336</v>
       </c>
-      <c r="Q9" s="6" t="n">
+      <c r="R9" s="6" t="n">
         <v>46310.291666666664</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:Q9"/>
+  <autoFilter ref="A6:R9"/>
   <mergeCells count="4">
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A4:Q4"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A4:R4"/>
   </mergeCells>
   <conditionalFormatting sqref="G7:G9">
     <cfRule type="expression" dxfId="5" priority="1">

</xml_diff>